<commit_message>
Add dropdown and conditional formatting to Excel output
</commit_message>
<xml_diff>
--- a/demo/test_spec.xlsx
+++ b/demo/test_spec.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="テスト仕様書" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="設定" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +29,20 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <sz val="10"/>
@@ -57,17 +62,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E75B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -112,30 +117,60 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="00808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00D9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="1"/>
+        <color rgb="00AAAAAA"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00EFEFEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -2519,6 +2554,185 @@
     <mergeCell ref="A12:L12"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>
+  <conditionalFormatting sqref="A15:L20">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$H15="完了"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>$H15="対象外"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A23:L29">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>$H23="完了"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>$H23="対象外"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A32:L34">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>$H32="完了"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="1">
+      <formula>$H32="対象外"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A37:L41">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>$H37="完了"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="1">
+      <formula>$H37="対象外"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A44:L46">
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>$H44="完了"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="1">
+      <formula>$H44="対象外"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A49:L50">
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>$H49="完了"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="1">
+      <formula>$H49="対象外"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A53:L54">
+    <cfRule type="expression" priority="13" dxfId="0">
+      <formula>$H53="完了"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="1">
+      <formula>$H53="対象外"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A57:L59">
+    <cfRule type="expression" priority="15" dxfId="0">
+      <formula>$H57="完了"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="1">
+      <formula>$H57="対象外"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="16">
+    <dataValidation sqref="H15:H20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="選択肢から選んでください：未着手 / 進行中 / 完了 / 対象外" type="list">
+      <formula1>"未着手,進行中,完了,対象外"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I15:I20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'設定'!$A$2:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="H23:H29" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="選択肢から選んでください：未着手 / 進行中 / 完了 / 対象外" type="list">
+      <formula1>"未着手,進行中,完了,対象外"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I23:I29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'設定'!$A$2:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="H32:H34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="選択肢から選んでください：未着手 / 進行中 / 完了 / 対象外" type="list">
+      <formula1>"未着手,進行中,完了,対象外"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I32:I34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'設定'!$A$2:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="H37:H41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="選択肢から選んでください：未着手 / 進行中 / 完了 / 対象外" type="list">
+      <formula1>"未着手,進行中,完了,対象外"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I37:I41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'設定'!$A$2:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="H44:H46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="選択肢から選んでください：未着手 / 進行中 / 完了 / 対象外" type="list">
+      <formula1>"未着手,進行中,完了,対象外"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I44:I46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'設定'!$A$2:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="H49:H50" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="選択肢から選んでください：未着手 / 進行中 / 完了 / 対象外" type="list">
+      <formula1>"未着手,進行中,完了,対象外"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I49:I50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'設定'!$A$2:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="H53:H54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="選択肢から選んでください：未着手 / 進行中 / 完了 / 対象外" type="list">
+      <formula1>"未着手,進行中,完了,対象外"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I53:I54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'設定'!$A$2:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="H57:H59" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="選択肢から選んでください：未着手 / 進行中 / 完了 / 対象外" type="list">
+      <formula1>"未着手,進行中,完了,対象外"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I57:I59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'設定'!$A$2:$A$6</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>担当者リスト</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>← 実際のメンバー名に変更してください</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>担当者A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>担当者B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>担当者C</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>担当者D</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>担当者E</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: change initial status from 未実施 to 未着手
</commit_message>
<xml_diff>
--- a/demo/test_spec.xlsx
+++ b/demo/test_spec.xlsx
@@ -745,7 +745,7 @@
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr"/>
@@ -787,7 +787,7 @@
       <c r="G16" s="5" t="inlineStr"/>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr"/>
@@ -829,7 +829,7 @@
       <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr"/>
@@ -871,7 +871,7 @@
       <c r="G18" s="5" t="inlineStr"/>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr"/>
@@ -913,7 +913,7 @@
       <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr"/>
@@ -955,7 +955,7 @@
       <c r="G20" s="5" t="inlineStr"/>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr"/>
@@ -1066,7 +1066,7 @@
       <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr"/>
@@ -1112,7 +1112,7 @@
       <c r="G24" s="5" t="inlineStr"/>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr"/>
@@ -1158,7 +1158,7 @@
       <c r="G25" s="4" t="inlineStr"/>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr"/>
@@ -1204,7 +1204,7 @@
       <c r="G26" s="5" t="inlineStr"/>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
       <c r="G27" s="4" t="inlineStr"/>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr"/>
@@ -1288,7 +1288,7 @@
       <c r="G28" s="5" t="inlineStr"/>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr"/>
@@ -1330,7 +1330,7 @@
       <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr"/>
@@ -1441,7 +1441,7 @@
       <c r="G32" s="4" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr"/>
@@ -1483,7 +1483,7 @@
       <c r="G33" s="5" t="inlineStr"/>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
@@ -1529,7 +1529,7 @@
       <c r="G34" s="4" t="inlineStr"/>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr"/>
@@ -1644,7 +1644,7 @@
       <c r="G37" s="4" t="inlineStr"/>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr"/>
@@ -1686,7 +1686,7 @@
       <c r="G38" s="5" t="inlineStr"/>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr"/>
@@ -1728,7 +1728,7 @@
       <c r="G39" s="4" t="inlineStr"/>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr"/>
@@ -1770,7 +1770,7 @@
       <c r="G40" s="5" t="inlineStr"/>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr"/>
@@ -1816,7 +1816,7 @@
       <c r="G41" s="4" t="inlineStr"/>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr"/>
@@ -1931,7 +1931,7 @@
       <c r="G44" s="4" t="inlineStr"/>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr"/>
@@ -1977,7 +1977,7 @@
       <c r="G45" s="5" t="inlineStr"/>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr"/>
@@ -2023,7 +2023,7 @@
       <c r="G46" s="4" t="inlineStr"/>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr"/>
@@ -2134,7 +2134,7 @@
       <c r="G49" s="4" t="inlineStr"/>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr"/>
@@ -2176,7 +2176,7 @@
       <c r="G50" s="5" t="inlineStr"/>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr"/>
@@ -2287,7 +2287,7 @@
       <c r="G53" s="4" t="inlineStr"/>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr"/>
@@ -2333,7 +2333,7 @@
       <c r="G54" s="5" t="inlineStr"/>
       <c r="H54" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       <c r="G57" s="4" t="inlineStr"/>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr"/>
@@ -2490,7 +2490,7 @@
       <c r="G58" s="5" t="inlineStr"/>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr"/>
@@ -2532,7 +2532,7 @@
       <c r="G59" s="4" t="inlineStr"/>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>未実施</t>
+          <t>未着手</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr"/>

</xml_diff>